<commit_message>
docs: update .gitignore with *.ps1 & *.bat
</commit_message>
<xml_diff>
--- a/.trash/易畫165與ASCII94.xlsx
+++ b/.trash/易畫165與ASCII94.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\share\git\rime-jek\.trash\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B69B784-A83C-4141-BAF9-25AFC67C1F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E691509-064E-4CEE-947D-2666F1DD8FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{B55F1E0F-6405-49D3-ACBC-C1F7C0B264EC}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="1124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="1126">
   <si>
     <t>268A</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -3735,6 +3735,14 @@
   </si>
   <si>
     <t>𝌂</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>𝌂𝌁</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>𝍂</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -13590,7 +13598,7 @@
         <v>1121</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>1122</v>
@@ -13599,6 +13607,9 @@
         <f>DEC2HEX(_xlfn.UNICODE(K21))</f>
         <v>1D301</v>
       </c>
+      <c r="M21" s="2" t="s">
+        <v>1124</v>
+      </c>
     </row>
     <row r="22" spans="1:20" ht="19.2">
       <c r="I22" s="2" t="s">
@@ -13624,6 +13635,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>